<commit_message>
Simulation, created class labels wrongly. Removed all output except smpbart dgp1 for some other check, will do later. Added DGP3 GP (not sure if correct, RF performs horribly). Remade DGP1 and DGP2. DGP2 and 3 data is added again, also for extranoise. RF output available for DGP2 variants and DGP3. Also removed waveform. DGP1 still need to choose version (with or without discontinuity) and run for all methods.
</commit_message>
<xml_diff>
--- a/output/rf_dgp2_output.xlsx
+++ b/output/rf_dgp2_output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5cac48941448979/Bureaublad/msc_thesis/thesis_code/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_42CED800ABA7AED2E87D25F7D01539EDE9E2BF29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4A9B5EA-DE1D-4248-9368-E39A3219E2A7}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED800246FE08C10EDAAE77C7623EDE9E2BF34" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4B03199-C042-40FC-B5DE-D0A04482D1C3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misclassification_rates" sheetId="1" r:id="rId1"/>
@@ -378,7 +378,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.249</v>
+        <v>0.251</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -388,42 +388,42 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.253</v>
+        <v>0.23699999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.26700000000000002</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.224</v>
+        <v>0.22700000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.27100000000000002</v>
+        <v>0.25600000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.26900000000000002</v>
+        <v>0.26400000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.26200000000000001</v>
+        <v>0.28699999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.26400000000000001</v>
+        <v>0.26700000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.26200000000000001</v>
+        <v>0.23699999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -432,7 +432,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.25560000000000005</v>
+        <v>0.25309999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -441,7 +441,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>1.5536337334705951E-2</v>
+        <v>1.9110497406166885E-2</v>
       </c>
     </row>
   </sheetData>
@@ -457,52 +457,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.379936728</v>
+        <v>0.34480968000000001</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.34906100800000001</v>
+        <v>0.34603995199999998</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.36454126399999998</v>
+        <v>0.36374101599999997</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.37865196800000001</v>
+        <v>0.377442744</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.36026957599999998</v>
+        <v>0.33039864000000002</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.36933172800000003</v>
+        <v>0.36281828799999999</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.37377956000000001</v>
+        <v>0.35288080799999999</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.387896464</v>
+        <v>0.39769267200000002</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.358822592</v>
+        <v>0.36939544000000002</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.38296758400000003</v>
+        <v>0.34311029599999998</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -511,7 +511,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.37052584720000004</v>
+        <v>0.3588329536</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -520,7 +520,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>1.2301120392122675E-2</v>
+        <v>1.9605536010024131E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>